<commit_message>
Scope playwright runs to the target JIRA ticket and add dashboard dev script
- orchestrator resolves specs from websites/<Site>/tests/<JIRA_ID>/ so
  `node scripts/orchestrate.js SCRUM-45` runs only SCRUM-45's UI+API specs
- move specs from tests/ into per-ticket folders under each website
- add framework (fixtures, config, pages, locators) for the POM layout
- add root `dev` script that starts the backend and Vite dashboard

Co-authored-by: CommandCodeBot <noreply@commandcode.ai>
</commit_message>
<xml_diff>
--- a/artifacts/SCRUM-32/SCRUM-32_TestCases.xlsx
+++ b/artifacts/SCRUM-32/SCRUM-32_TestCases.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="87">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -63,7 +63,7 @@
     <t>The application loads successfully and is accessible.</t>
   </si>
   <si>
-    <t>Test passed successfully.</t>
+    <t/>
   </si>
   <si>
     <t>High</t>
@@ -75,10 +75,7 @@
     <t>Automated</t>
   </si>
   <si>
-    <t>Pass</t>
-  </si>
-  <si>
-    <t/>
+    <t>Not Run</t>
   </si>
   <si>
     <t>TC_UI_02</t>
@@ -335,9 +332,6 @@
     <t>The page content is rendered and visible.</t>
   </si>
   <si>
-    <t>Not Run</t>
-  </si>
-  <si>
     <t>TC_UI_BUG</t>
   </si>
   <si>
@@ -359,7 +353,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -370,10 +364,6 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FF22C55E"/>
     </font>
   </fonts>
   <fills count="3">
@@ -424,7 +414,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -847,31 +837,31 @@
         <v>20</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" ht="100" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>26</v>
-      </c>
       <c r="H3" s="2" t="s">
         <v>18</v>
       </c>
@@ -882,30 +872,30 @@
         <v>20</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" ht="100" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>30</v>
-      </c>
       <c r="F4" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>18</v>
@@ -917,30 +907,30 @@
         <v>20</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" ht="115" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>34</v>
-      </c>
       <c r="F5" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>18</v>
@@ -952,30 +942,30 @@
         <v>20</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" ht="85" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="F6" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>18</v>
@@ -987,30 +977,30 @@
         <v>20</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" ht="100" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="F7" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>18</v>
@@ -1022,30 +1012,30 @@
         <v>20</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" ht="100" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>46</v>
-      </c>
       <c r="F8" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>18</v>
@@ -1057,30 +1047,30 @@
         <v>20</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" ht="100" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>50</v>
-      </c>
       <c r="F9" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>18</v>
@@ -1092,30 +1082,30 @@
         <v>20</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" ht="100" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>54</v>
-      </c>
       <c r="F10" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>18</v>
@@ -1127,30 +1117,30 @@
         <v>20</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" ht="100" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>58</v>
-      </c>
       <c r="F11" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>18</v>
@@ -1162,30 +1152,30 @@
         <v>20</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" ht="100" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="E12" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E12" s="2" t="s">
-        <v>62</v>
-      </c>
       <c r="F12" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>18</v>
@@ -1197,30 +1187,30 @@
         <v>20</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" ht="85" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="E13" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="E13" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="F13" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>18</v>
@@ -1232,30 +1222,30 @@
         <v>20</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" ht="100" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="E14" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="E14" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="F14" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>18</v>
@@ -1267,30 +1257,30 @@
         <v>20</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" ht="100" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="E15" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="F15" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>18</v>
@@ -1302,30 +1292,30 @@
         <v>20</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" ht="100" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="E16" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="E16" s="2" t="s">
-        <v>78</v>
-      </c>
       <c r="F16" s="2" t="s">
         <v>16</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>18</v>
@@ -1337,30 +1327,30 @@
         <v>20</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17" ht="55" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C17" s="2" t="s">
+      <c r="D17" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>82</v>
-      </c>
       <c r="F17" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>18</v>
@@ -1369,34 +1359,34 @@
         <v>19</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>83</v>
+        <v>20</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="18" ht="55" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D18" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C18" s="2" t="s">
+      <c r="E18" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="F18" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E18" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>88</v>
-      </c>
       <c r="H18" s="2" t="s">
         <v>18</v>
       </c>
@@ -1404,14 +1394,14 @@
         <v>19</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>83</v>
+        <v>20</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>